<commit_message>
results(Q1): rerun verified plan under interface power cap
Refresh result1.xlsx, Table 1/2, metrics, and figures after moving the 5000 kW limit to the microgrid interface. Daily cost is 35126.95 yuan.

Co-authored-by: Sen-illion <Sen-illion@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/results/Q1/result1.xlsx
+++ b/results/Q1/result1.xlsx
@@ -470,57 +470,57 @@
     <row r="2" ht="14" customHeight="1">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>0:10-0:20</t>
+          <t>00:00-00:10</t>
         </is>
       </c>
       <c r="B2" s="7" t="n">
-        <v>1499.2337</v>
+        <v>1406.6411</v>
       </c>
     </row>
     <row r="3" ht="14" customHeight="1">
       <c r="A3" s="5" t="inlineStr">
         <is>
-          <t>0:20-0:30</t>
+          <t>00:10-00:20</t>
         </is>
       </c>
       <c r="B3" s="7" t="n">
-        <v>1498.9225</v>
+        <v>1406.3299</v>
       </c>
     </row>
     <row r="4" ht="14" customHeight="1">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>0:30-0:40</t>
+          <t>00:20-00:30</t>
         </is>
       </c>
       <c r="B4" s="7" t="n">
-        <v>1499.9764</v>
+        <v>1407.3838</v>
       </c>
     </row>
     <row r="5" ht="14" customHeight="1">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>0:40-0:50</t>
+          <t>00:30-00:40</t>
         </is>
       </c>
       <c r="B5" s="7" t="n">
-        <v>1279.4443</v>
+        <v>1409.0739</v>
       </c>
     </row>
     <row r="6" ht="14" customHeight="1">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>0:50-1:00</t>
+          <t>00:40-00:50</t>
         </is>
       </c>
       <c r="B6" s="7" t="n">
-        <v>1502.3971</v>
+        <v>1409.8045</v>
       </c>
     </row>
     <row r="7" ht="14" customHeight="1">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>1:00-1:10</t>
+          <t>00:50-01:00</t>
         </is>
       </c>
       <c r="B7" s="7" t="n">
@@ -530,7 +530,7 @@
     <row r="8" ht="14" customHeight="1">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>1:10-1:20</t>
+          <t>01:00-01:10</t>
         </is>
       </c>
       <c r="B8" s="7" t="n">
@@ -540,7 +540,7 @@
     <row r="9" ht="14" customHeight="1">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>1:20-1:30</t>
+          <t>01:10-01:20</t>
         </is>
       </c>
       <c r="B9" s="7" t="n">
@@ -550,17 +550,17 @@
     <row r="10" ht="14" customHeight="1">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>1:30-1:40</t>
+          <t>01:20-01:30</t>
         </is>
       </c>
       <c r="B10" s="7" t="n">
-        <v>577.82805</v>
+        <v>911.16138</v>
       </c>
     </row>
     <row r="11" ht="14" customHeight="1">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>1:40-1:50</t>
+          <t>01:30-01:40</t>
         </is>
       </c>
       <c r="B11" s="7" t="n">
@@ -570,7 +570,7 @@
     <row r="12" ht="14" customHeight="1">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>1:50-2:00</t>
+          <t>01:40-01:50</t>
         </is>
       </c>
       <c r="B12" s="7" t="n">
@@ -580,7 +580,7 @@
     <row r="13" ht="14" customHeight="1">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>2:00-2:10</t>
+          <t>01:50-02:00</t>
         </is>
       </c>
       <c r="B13" s="7" t="n">
@@ -590,7 +590,7 @@
     <row r="14" ht="14" customHeight="1">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>2:10-2:20</t>
+          <t>02:00-02:10</t>
         </is>
       </c>
       <c r="B14" s="7" t="n">
@@ -600,7 +600,7 @@
     <row r="15" ht="14" customHeight="1">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>2:20-2:30</t>
+          <t>02:10-02:20</t>
         </is>
       </c>
       <c r="B15" s="7" t="n">
@@ -610,7 +610,7 @@
     <row r="16" ht="14" customHeight="1">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>2:30-2:40</t>
+          <t>02:20-02:30</t>
         </is>
       </c>
       <c r="B16" s="7" t="n">
@@ -620,7 +620,7 @@
     <row r="17" ht="14" customHeight="1">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>2:40-2:50</t>
+          <t>02:30-02:40</t>
         </is>
       </c>
       <c r="B17" s="7" t="n">
@@ -630,7 +630,7 @@
     <row r="18" ht="14" customHeight="1">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>2:50-3:00</t>
+          <t>02:40-02:50</t>
         </is>
       </c>
       <c r="B18" s="7" t="n">
@@ -640,7 +640,7 @@
     <row r="19" ht="14" customHeight="1">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>3:00-3:10</t>
+          <t>02:50-03:00</t>
         </is>
       </c>
       <c r="B19" s="7" t="n">
@@ -650,7 +650,7 @@
     <row r="20" ht="14" customHeight="1">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t>3:10-3:20</t>
+          <t>03:00-03:10</t>
         </is>
       </c>
       <c r="B20" s="7" t="n">
@@ -660,7 +660,7 @@
     <row r="21" ht="14" customHeight="1">
       <c r="A21" s="5" t="inlineStr">
         <is>
-          <t>3:20-3:30</t>
+          <t>03:10-03:20</t>
         </is>
       </c>
       <c r="B21" s="7" t="n">
@@ -670,7 +670,7 @@
     <row r="22" ht="14" customHeight="1">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>3:30-3:40</t>
+          <t>03:20-03:30</t>
         </is>
       </c>
       <c r="B22" s="7" t="n">
@@ -680,7 +680,7 @@
     <row r="23" ht="14" customHeight="1">
       <c r="A23" s="5" t="inlineStr">
         <is>
-          <t>3:40-3:50</t>
+          <t>03:30-03:40</t>
         </is>
       </c>
       <c r="B23" s="7" t="n">
@@ -690,7 +690,7 @@
     <row r="24" ht="14" customHeight="1">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>3:50-4:00</t>
+          <t>03:40-03:50</t>
         </is>
       </c>
       <c r="B24" s="7" t="n">
@@ -700,7 +700,7 @@
     <row r="25" ht="14" customHeight="1">
       <c r="A25" s="5" t="inlineStr">
         <is>
-          <t>4:00-4:10</t>
+          <t>03:50-04:00</t>
         </is>
       </c>
       <c r="B25" s="7" t="n">
@@ -710,7 +710,7 @@
     <row r="26" ht="14" customHeight="1">
       <c r="A26" s="5" t="inlineStr">
         <is>
-          <t>4:10-4:20</t>
+          <t>04:00-04:10</t>
         </is>
       </c>
       <c r="B26" s="7" t="n">
@@ -720,7 +720,7 @@
     <row r="27" ht="14" customHeight="1">
       <c r="A27" s="5" t="inlineStr">
         <is>
-          <t>4:20-4:30</t>
+          <t>04:10-04:20</t>
         </is>
       </c>
       <c r="B27" s="7" t="n">
@@ -730,7 +730,7 @@
     <row r="28" ht="14" customHeight="1">
       <c r="A28" s="5" t="inlineStr">
         <is>
-          <t>4:30-4:40</t>
+          <t>04:20-04:30</t>
         </is>
       </c>
       <c r="B28" s="7" t="n">
@@ -740,7 +740,7 @@
     <row r="29" ht="14" customHeight="1">
       <c r="A29" s="5" t="inlineStr">
         <is>
-          <t>4:40-4:50</t>
+          <t>04:30-04:40</t>
         </is>
       </c>
       <c r="B29" s="7" t="n">
@@ -750,7 +750,7 @@
     <row r="30" ht="14" customHeight="1">
       <c r="A30" s="5" t="inlineStr">
         <is>
-          <t>4:50-5:00</t>
+          <t>04:40-04:50</t>
         </is>
       </c>
       <c r="B30" s="7" t="n">
@@ -760,7 +760,7 @@
     <row r="31" ht="14" customHeight="1">
       <c r="A31" s="5" t="inlineStr">
         <is>
-          <t>5:00-5:10</t>
+          <t>04:50-05:00</t>
         </is>
       </c>
       <c r="B31" s="7" t="n">
@@ -770,7 +770,7 @@
     <row r="32" ht="14" customHeight="1">
       <c r="A32" s="5" t="inlineStr">
         <is>
-          <t>5:10-5:20</t>
+          <t>05:00-05:10</t>
         </is>
       </c>
       <c r="B32" s="7" t="n">
@@ -780,7 +780,7 @@
     <row r="33" ht="14" customHeight="1">
       <c r="A33" s="5" t="inlineStr">
         <is>
-          <t>5:20-5:30</t>
+          <t>05:10-05:20</t>
         </is>
       </c>
       <c r="B33" s="7" t="n">
@@ -790,7 +790,7 @@
     <row r="34" ht="14" customHeight="1">
       <c r="A34" s="5" t="inlineStr">
         <is>
-          <t>5:30-5:40</t>
+          <t>05:20-05:30</t>
         </is>
       </c>
       <c r="B34" s="7" t="n">
@@ -800,17 +800,17 @@
     <row r="35" ht="14" customHeight="1">
       <c r="A35" s="5" t="inlineStr">
         <is>
-          <t>5:40-5:50</t>
+          <t>05:30-05:40</t>
         </is>
       </c>
       <c r="B35" s="7" t="n">
-        <v>1476.2524</v>
+        <v>1383.6598</v>
       </c>
     </row>
     <row r="36" ht="14" customHeight="1">
       <c r="A36" s="5" t="inlineStr">
         <is>
-          <t>5:50-6:00</t>
+          <t>05:40-05:50</t>
         </is>
       </c>
       <c r="B36" s="7" t="n">
@@ -820,7 +820,7 @@
     <row r="37" ht="14" customHeight="1">
       <c r="A37" s="5" t="inlineStr">
         <is>
-          <t>6:00-6:10</t>
+          <t>05:50-06:00</t>
         </is>
       </c>
       <c r="B37" s="7" t="n">
@@ -830,7 +830,7 @@
     <row r="38" ht="14" customHeight="1">
       <c r="A38" s="5" t="inlineStr">
         <is>
-          <t>6:10-6:20</t>
+          <t>06:00-06:10</t>
         </is>
       </c>
       <c r="B38" s="7" t="n">
@@ -840,7 +840,7 @@
     <row r="39" ht="14" customHeight="1">
       <c r="A39" s="5" t="inlineStr">
         <is>
-          <t>6:20-6:30</t>
+          <t>06:10-06:20</t>
         </is>
       </c>
       <c r="B39" s="7" t="n">
@@ -850,7 +850,7 @@
     <row r="40" ht="14" customHeight="1">
       <c r="A40" s="5" t="inlineStr">
         <is>
-          <t>6:30-6:40</t>
+          <t>06:20-06:30</t>
         </is>
       </c>
       <c r="B40" s="7" t="n">
@@ -860,7 +860,7 @@
     <row r="41" ht="14" customHeight="1">
       <c r="A41" s="5" t="inlineStr">
         <is>
-          <t>6:40-6:50</t>
+          <t>06:30-06:40</t>
         </is>
       </c>
       <c r="B41" s="7" t="n">
@@ -870,7 +870,7 @@
     <row r="42" ht="14" customHeight="1">
       <c r="A42" s="5" t="inlineStr">
         <is>
-          <t>6:50-7:00</t>
+          <t>06:40-06:50</t>
         </is>
       </c>
       <c r="B42" s="7" t="n">
@@ -880,7 +880,7 @@
     <row r="43" ht="14" customHeight="1">
       <c r="A43" s="5" t="inlineStr">
         <is>
-          <t>7:00-7:10</t>
+          <t>06:50-07:00</t>
         </is>
       </c>
       <c r="B43" s="7" t="n">
@@ -890,7 +890,7 @@
     <row r="44" ht="14" customHeight="1">
       <c r="A44" s="5" t="inlineStr">
         <is>
-          <t>7:10-7:20</t>
+          <t>07:00-07:10</t>
         </is>
       </c>
       <c r="B44" s="7" t="n">
@@ -900,7 +900,7 @@
     <row r="45" ht="14" customHeight="1">
       <c r="A45" s="5" t="inlineStr">
         <is>
-          <t>7:20-7:30</t>
+          <t>07:10-07:20</t>
         </is>
       </c>
       <c r="B45" s="7" t="n">
@@ -910,7 +910,7 @@
     <row r="46" ht="14" customHeight="1">
       <c r="A46" s="5" t="inlineStr">
         <is>
-          <t>7:30-7:40</t>
+          <t>07:20-07:30</t>
         </is>
       </c>
       <c r="B46" s="7" t="n">
@@ -920,7 +920,7 @@
     <row r="47" ht="14" customHeight="1">
       <c r="A47" s="5" t="inlineStr">
         <is>
-          <t>7:40-7:50</t>
+          <t>07:30-07:40</t>
         </is>
       </c>
       <c r="B47" s="7" t="n">
@@ -930,7 +930,7 @@
     <row r="48" ht="14" customHeight="1">
       <c r="A48" s="5" t="inlineStr">
         <is>
-          <t>7:50-8:00</t>
+          <t>07:40-07:50</t>
         </is>
       </c>
       <c r="B48" s="7" t="n">
@@ -940,7 +940,7 @@
     <row r="49" ht="14" customHeight="1">
       <c r="A49" s="5" t="inlineStr">
         <is>
-          <t>8:00-8:10</t>
+          <t>07:50-08:00</t>
         </is>
       </c>
       <c r="B49" s="7" t="n">
@@ -950,7 +950,7 @@
     <row r="50" ht="14" customHeight="1">
       <c r="A50" s="5" t="inlineStr">
         <is>
-          <t>8:10-8:20</t>
+          <t>08:00-08:10</t>
         </is>
       </c>
       <c r="B50" s="7" t="n">
@@ -960,7 +960,7 @@
     <row r="51" ht="14" customHeight="1">
       <c r="A51" s="5" t="inlineStr">
         <is>
-          <t>8:20-8:30</t>
+          <t>08:10-08:20</t>
         </is>
       </c>
       <c r="B51" s="7" t="n">
@@ -970,7 +970,7 @@
     <row r="52" ht="14" customHeight="1">
       <c r="A52" s="5" t="inlineStr">
         <is>
-          <t>8:30-8:40</t>
+          <t>08:20-08:30</t>
         </is>
       </c>
       <c r="B52" s="7" t="n">
@@ -980,7 +980,7 @@
     <row r="53" ht="14" customHeight="1">
       <c r="A53" s="5" t="inlineStr">
         <is>
-          <t>8:40-8:50</t>
+          <t>08:30-08:40</t>
         </is>
       </c>
       <c r="B53" s="7" t="n">
@@ -990,7 +990,7 @@
     <row r="54" ht="14" customHeight="1">
       <c r="A54" s="5" t="inlineStr">
         <is>
-          <t>8:50-9:00</t>
+          <t>08:40-08:50</t>
         </is>
       </c>
       <c r="B54" s="7" t="n">
@@ -1000,7 +1000,7 @@
     <row r="55" ht="14" customHeight="1">
       <c r="A55" s="5" t="inlineStr">
         <is>
-          <t>9:00-9:10</t>
+          <t>08:50-09:00</t>
         </is>
       </c>
       <c r="B55" s="7" t="n">
@@ -1010,7 +1010,7 @@
     <row r="56" ht="14" customHeight="1">
       <c r="A56" s="5" t="inlineStr">
         <is>
-          <t>9:10-9:20</t>
+          <t>09:00-09:10</t>
         </is>
       </c>
       <c r="B56" s="7" t="n">
@@ -1020,7 +1020,7 @@
     <row r="57" ht="14" customHeight="1">
       <c r="A57" s="5" t="inlineStr">
         <is>
-          <t>9:20-9:30</t>
+          <t>09:10-09:20</t>
         </is>
       </c>
       <c r="B57" s="7" t="n">
@@ -1030,7 +1030,7 @@
     <row r="58" ht="14" customHeight="1">
       <c r="A58" s="5" t="inlineStr">
         <is>
-          <t>9:30-9:40</t>
+          <t>09:20-09:30</t>
         </is>
       </c>
       <c r="B58" s="7" t="n">
@@ -1040,7 +1040,7 @@
     <row r="59" ht="14" customHeight="1">
       <c r="A59" s="5" t="inlineStr">
         <is>
-          <t>9:40-9:50</t>
+          <t>09:30-09:40</t>
         </is>
       </c>
       <c r="B59" s="7" t="n">
@@ -1050,7 +1050,7 @@
     <row r="60" ht="14" customHeight="1">
       <c r="A60" s="5" t="inlineStr">
         <is>
-          <t>9:50-10:00</t>
+          <t>09:40-09:50</t>
         </is>
       </c>
       <c r="B60" s="7" t="n">
@@ -1060,7 +1060,7 @@
     <row r="61" ht="14" customHeight="1">
       <c r="A61" s="5" t="inlineStr">
         <is>
-          <t>10:00-10:10</t>
+          <t>09:50-10:00</t>
         </is>
       </c>
       <c r="B61" s="7" t="n">
@@ -1070,7 +1070,7 @@
     <row r="62" ht="14" customHeight="1">
       <c r="A62" s="5" t="inlineStr">
         <is>
-          <t>10:10-10:20</t>
+          <t>10:00-10:10</t>
         </is>
       </c>
       <c r="B62" s="7" t="n">
@@ -1080,7 +1080,7 @@
     <row r="63" ht="14" customHeight="1">
       <c r="A63" s="5" t="inlineStr">
         <is>
-          <t>10:20-10:30</t>
+          <t>10:10-10:20</t>
         </is>
       </c>
       <c r="B63" s="7" t="n">
@@ -1090,7 +1090,7 @@
     <row r="64" ht="14" customHeight="1">
       <c r="A64" s="5" t="inlineStr">
         <is>
-          <t>10:30-10:40</t>
+          <t>10:20-10:30</t>
         </is>
       </c>
       <c r="B64" s="7" t="n">
@@ -1100,7 +1100,7 @@
     <row r="65" ht="14" customHeight="1">
       <c r="A65" s="5" t="inlineStr">
         <is>
-          <t>10:40-10:50</t>
+          <t>10:30-10:40</t>
         </is>
       </c>
       <c r="B65" s="7" t="n">
@@ -1110,7 +1110,7 @@
     <row r="66" ht="14" customHeight="1">
       <c r="A66" s="5" t="inlineStr">
         <is>
-          <t>10:50-11:00</t>
+          <t>10:40-10:50</t>
         </is>
       </c>
       <c r="B66" s="7" t="n">
@@ -1120,7 +1120,7 @@
     <row r="67" ht="14" customHeight="1">
       <c r="A67" s="5" t="inlineStr">
         <is>
-          <t>11:00-11:10</t>
+          <t>10:50-11:00</t>
         </is>
       </c>
       <c r="B67" s="7" t="n">
@@ -1130,17 +1130,17 @@
     <row r="68" ht="14" customHeight="1">
       <c r="A68" s="5" t="inlineStr">
         <is>
-          <t>11:10-11:20</t>
+          <t>11:00-11:10</t>
         </is>
       </c>
       <c r="B68" s="7" t="n">
-        <v>667.76351</v>
+        <v>575.17092</v>
       </c>
     </row>
     <row r="69" ht="14" customHeight="1">
       <c r="A69" s="5" t="inlineStr">
         <is>
-          <t>11:20-11:30</t>
+          <t>11:10-11:20</t>
         </is>
       </c>
       <c r="B69" s="7" t="n">
@@ -1150,7 +1150,7 @@
     <row r="70" ht="14" customHeight="1">
       <c r="A70" s="5" t="inlineStr">
         <is>
-          <t>11:30-11:40</t>
+          <t>11:20-11:30</t>
         </is>
       </c>
       <c r="B70" s="7" t="n">
@@ -1160,77 +1160,77 @@
     <row r="71" ht="14" customHeight="1">
       <c r="A71" s="5" t="inlineStr">
         <is>
-          <t>11:40-11:50</t>
+          <t>11:30-11:40</t>
         </is>
       </c>
       <c r="B71" s="7" t="n">
-        <v>0</v>
+        <v>179.27717</v>
       </c>
     </row>
     <row r="72" ht="14" customHeight="1">
       <c r="A72" s="5" t="inlineStr">
         <is>
-          <t>11:50-12:00</t>
+          <t>11:40-11:50</t>
         </is>
       </c>
       <c r="B72" s="7" t="n">
-        <v>143.84613</v>
+        <v>520.12452</v>
       </c>
     </row>
     <row r="73" ht="14" customHeight="1">
       <c r="A73" s="5" t="inlineStr">
         <is>
-          <t>12:00-12:10</t>
+          <t>11:50-12:00</t>
         </is>
       </c>
       <c r="B73" s="7" t="n">
-        <v>578.99549</v>
+        <v>486.4029</v>
       </c>
     </row>
     <row r="74" ht="14" customHeight="1">
       <c r="A74" s="5" t="inlineStr">
         <is>
-          <t>12:10-12:20</t>
+          <t>12:00-12:10</t>
         </is>
       </c>
       <c r="B74" s="7" t="n">
-        <v>573.00504</v>
+        <v>480.41245</v>
       </c>
     </row>
     <row r="75" ht="14" customHeight="1">
       <c r="A75" s="5" t="inlineStr">
         <is>
-          <t>12:20-12:30</t>
+          <t>12:10-12:20</t>
         </is>
       </c>
       <c r="B75" s="7" t="n">
-        <v>577.89259</v>
+        <v>485.3</v>
       </c>
     </row>
     <row r="76" ht="14" customHeight="1">
       <c r="A76" s="5" t="inlineStr">
         <is>
-          <t>12:30-12:40</t>
+          <t>12:20-12:30</t>
         </is>
       </c>
       <c r="B76" s="7" t="n">
-        <v>581.19956</v>
+        <v>488.60697</v>
       </c>
     </row>
     <row r="77" ht="14" customHeight="1">
       <c r="A77" s="5" t="inlineStr">
         <is>
-          <t>12:40-12:50</t>
+          <t>12:30-12:40</t>
         </is>
       </c>
       <c r="B77" s="7" t="n">
-        <v>590.86333</v>
+        <v>498.27073</v>
       </c>
     </row>
     <row r="78" ht="14" customHeight="1">
       <c r="A78" s="5" t="inlineStr">
         <is>
-          <t>12:50-13:00</t>
+          <t>12:40-12:50</t>
         </is>
       </c>
       <c r="B78" s="7" t="n">
@@ -1240,7 +1240,7 @@
     <row r="79" ht="14" customHeight="1">
       <c r="A79" s="5" t="inlineStr">
         <is>
-          <t>13:00-13:10</t>
+          <t>12:50-13:00</t>
         </is>
       </c>
       <c r="B79" s="7" t="n">
@@ -1250,7 +1250,7 @@
     <row r="80" ht="14" customHeight="1">
       <c r="A80" s="5" t="inlineStr">
         <is>
-          <t>13:10-13:20</t>
+          <t>13:00-13:10</t>
         </is>
       </c>
       <c r="B80" s="7" t="n">
@@ -1260,7 +1260,7 @@
     <row r="81" ht="14" customHeight="1">
       <c r="A81" s="5" t="inlineStr">
         <is>
-          <t>13:20-13:30</t>
+          <t>13:10-13:20</t>
         </is>
       </c>
       <c r="B81" s="7" t="n">
@@ -1270,7 +1270,7 @@
     <row r="82" ht="14" customHeight="1">
       <c r="A82" s="5" t="inlineStr">
         <is>
-          <t>13:30-13:40</t>
+          <t>13:20-13:30</t>
         </is>
       </c>
       <c r="B82" s="7" t="n">
@@ -1280,7 +1280,7 @@
     <row r="83" ht="14" customHeight="1">
       <c r="A83" s="5" t="inlineStr">
         <is>
-          <t>13:40-13:50</t>
+          <t>13:30-13:40</t>
         </is>
       </c>
       <c r="B83" s="7" t="n">
@@ -1290,7 +1290,7 @@
     <row r="84" ht="14" customHeight="1">
       <c r="A84" s="5" t="inlineStr">
         <is>
-          <t>13:50-14:00</t>
+          <t>13:40-13:50</t>
         </is>
       </c>
       <c r="B84" s="7" t="n">
@@ -1300,7 +1300,7 @@
     <row r="85" ht="14" customHeight="1">
       <c r="A85" s="5" t="inlineStr">
         <is>
-          <t>14:00-14:10</t>
+          <t>13:50-14:00</t>
         </is>
       </c>
       <c r="B85" s="7" t="n">
@@ -1310,7 +1310,7 @@
     <row r="86" ht="14" customHeight="1">
       <c r="A86" s="5" t="inlineStr">
         <is>
-          <t>14:10-14:20</t>
+          <t>14:00-14:10</t>
         </is>
       </c>
       <c r="B86" s="7" t="n">
@@ -1320,7 +1320,7 @@
     <row r="87" ht="14" customHeight="1">
       <c r="A87" s="5" t="inlineStr">
         <is>
-          <t>14:20-14:30</t>
+          <t>14:10-14:20</t>
         </is>
       </c>
       <c r="B87" s="7" t="n">
@@ -1330,7 +1330,7 @@
     <row r="88" ht="14" customHeight="1">
       <c r="A88" s="5" t="inlineStr">
         <is>
-          <t>14:30-14:40</t>
+          <t>14:20-14:30</t>
         </is>
       </c>
       <c r="B88" s="7" t="n">
@@ -1340,7 +1340,7 @@
     <row r="89" ht="14" customHeight="1">
       <c r="A89" s="5" t="inlineStr">
         <is>
-          <t>14:40-14:50</t>
+          <t>14:30-14:40</t>
         </is>
       </c>
       <c r="B89" s="7" t="n">
@@ -1350,7 +1350,7 @@
     <row r="90" ht="14" customHeight="1">
       <c r="A90" s="5" t="inlineStr">
         <is>
-          <t>14:50-15:00</t>
+          <t>14:40-14:50</t>
         </is>
       </c>
       <c r="B90" s="7" t="n">
@@ -1360,7 +1360,7 @@
     <row r="91" ht="14" customHeight="1">
       <c r="A91" s="5" t="inlineStr">
         <is>
-          <t>15:00-15:10</t>
+          <t>14:50-15:00</t>
         </is>
       </c>
       <c r="B91" s="7" t="n">
@@ -1370,7 +1370,7 @@
     <row r="92" ht="14" customHeight="1">
       <c r="A92" s="5" t="inlineStr">
         <is>
-          <t>15:10-15:20</t>
+          <t>15:00-15:10</t>
         </is>
       </c>
       <c r="B92" s="7" t="n">
@@ -1380,7 +1380,7 @@
     <row r="93" ht="14" customHeight="1">
       <c r="A93" s="5" t="inlineStr">
         <is>
-          <t>15:20-15:30</t>
+          <t>15:10-15:20</t>
         </is>
       </c>
       <c r="B93" s="7" t="n">
@@ -1390,7 +1390,7 @@
     <row r="94" ht="14" customHeight="1">
       <c r="A94" s="5" t="inlineStr">
         <is>
-          <t>15:30-15:40</t>
+          <t>15:20-15:30</t>
         </is>
       </c>
       <c r="B94" s="7" t="n">
@@ -1400,7 +1400,7 @@
     <row r="95" ht="14" customHeight="1">
       <c r="A95" s="5" t="inlineStr">
         <is>
-          <t>15:40-15:50</t>
+          <t>15:30-15:40</t>
         </is>
       </c>
       <c r="B95" s="7" t="n">
@@ -1410,7 +1410,7 @@
     <row r="96" ht="14" customHeight="1">
       <c r="A96" s="5" t="inlineStr">
         <is>
-          <t>15:50-16:00</t>
+          <t>15:40-15:50</t>
         </is>
       </c>
       <c r="B96" s="7" t="n">
@@ -1420,7 +1420,7 @@
     <row r="97" ht="14" customHeight="1">
       <c r="A97" s="5" t="inlineStr">
         <is>
-          <t>16:00-16:10</t>
+          <t>15:50-16:00</t>
         </is>
       </c>
       <c r="B97" s="7" t="n">
@@ -1430,7 +1430,7 @@
     <row r="98" ht="14" customHeight="1">
       <c r="A98" s="5" t="inlineStr">
         <is>
-          <t>16:10-16:20</t>
+          <t>16:00-16:10</t>
         </is>
       </c>
       <c r="B98" s="7" t="n">
@@ -1440,7 +1440,7 @@
     <row r="99" ht="14" customHeight="1">
       <c r="A99" s="5" t="inlineStr">
         <is>
-          <t>16:20-16:30</t>
+          <t>16:10-16:20</t>
         </is>
       </c>
       <c r="B99" s="7" t="n">
@@ -1450,7 +1450,7 @@
     <row r="100" ht="14" customHeight="1">
       <c r="A100" s="5" t="inlineStr">
         <is>
-          <t>16:30-16:40</t>
+          <t>16:20-16:30</t>
         </is>
       </c>
       <c r="B100" s="7" t="n">
@@ -1460,7 +1460,7 @@
     <row r="101" ht="14" customHeight="1">
       <c r="A101" s="5" t="inlineStr">
         <is>
-          <t>16:40-16:50</t>
+          <t>16:30-16:40</t>
         </is>
       </c>
       <c r="B101" s="7" t="n">
@@ -1470,7 +1470,7 @@
     <row r="102" ht="14" customHeight="1">
       <c r="A102" s="5" t="inlineStr">
         <is>
-          <t>16:50-17:00</t>
+          <t>16:40-16:50</t>
         </is>
       </c>
       <c r="B102" s="7" t="n">
@@ -1480,7 +1480,7 @@
     <row r="103" ht="14" customHeight="1">
       <c r="A103" s="5" t="inlineStr">
         <is>
-          <t>17:00-17:10</t>
+          <t>16:50-17:00</t>
         </is>
       </c>
       <c r="B103" s="7" t="n">
@@ -1490,7 +1490,7 @@
     <row r="104" ht="14" customHeight="1">
       <c r="A104" s="5" t="inlineStr">
         <is>
-          <t>17:10-17:20</t>
+          <t>17:00-17:10</t>
         </is>
       </c>
       <c r="B104" s="7" t="n">
@@ -1500,7 +1500,7 @@
     <row r="105" ht="14" customHeight="1">
       <c r="A105" s="5" t="inlineStr">
         <is>
-          <t>17:20-17:30</t>
+          <t>17:10-17:20</t>
         </is>
       </c>
       <c r="B105" s="7" t="n">
@@ -1510,7 +1510,7 @@
     <row r="106" ht="14" customHeight="1">
       <c r="A106" s="5" t="inlineStr">
         <is>
-          <t>17:30-17:40</t>
+          <t>17:20-17:30</t>
         </is>
       </c>
       <c r="B106" s="7" t="n">
@@ -1520,7 +1520,7 @@
     <row r="107" ht="14" customHeight="1">
       <c r="A107" s="5" t="inlineStr">
         <is>
-          <t>17:40-17:50</t>
+          <t>17:30-17:40</t>
         </is>
       </c>
       <c r="B107" s="7" t="n">
@@ -1530,7 +1530,7 @@
     <row r="108" ht="14" customHeight="1">
       <c r="A108" s="5" t="inlineStr">
         <is>
-          <t>17:50-18:00</t>
+          <t>17:40-17:50</t>
         </is>
       </c>
       <c r="B108" s="7" t="n">
@@ -1540,7 +1540,7 @@
     <row r="109" ht="14" customHeight="1">
       <c r="A109" s="5" t="inlineStr">
         <is>
-          <t>18:00-18:10</t>
+          <t>17:50-18:00</t>
         </is>
       </c>
       <c r="B109" s="7" t="n">
@@ -1550,7 +1550,7 @@
     <row r="110" ht="14" customHeight="1">
       <c r="A110" s="5" t="inlineStr">
         <is>
-          <t>18:10-18:20</t>
+          <t>18:00-18:10</t>
         </is>
       </c>
       <c r="B110" s="7" t="n">
@@ -1560,7 +1560,7 @@
     <row r="111" ht="14" customHeight="1">
       <c r="A111" s="5" t="inlineStr">
         <is>
-          <t>18:20-18:30</t>
+          <t>18:10-18:20</t>
         </is>
       </c>
       <c r="B111" s="7" t="n">
@@ -1570,7 +1570,7 @@
     <row r="112" ht="14" customHeight="1">
       <c r="A112" s="5" t="inlineStr">
         <is>
-          <t>18:30-18:40</t>
+          <t>18:20-18:30</t>
         </is>
       </c>
       <c r="B112" s="7" t="n">
@@ -1580,7 +1580,7 @@
     <row r="113" ht="14" customHeight="1">
       <c r="A113" s="5" t="inlineStr">
         <is>
-          <t>18:40-18:50</t>
+          <t>18:30-18:40</t>
         </is>
       </c>
       <c r="B113" s="7" t="n">
@@ -1590,7 +1590,7 @@
     <row r="114" ht="14" customHeight="1">
       <c r="A114" s="5" t="inlineStr">
         <is>
-          <t>18:50-19:00</t>
+          <t>18:40-18:50</t>
         </is>
       </c>
       <c r="B114" s="7" t="n">
@@ -1600,7 +1600,7 @@
     <row r="115" ht="14" customHeight="1">
       <c r="A115" s="5" t="inlineStr">
         <is>
-          <t>19:00-19:10</t>
+          <t>18:50-19:00</t>
         </is>
       </c>
       <c r="B115" s="7" t="n">
@@ -1610,7 +1610,7 @@
     <row r="116" ht="14" customHeight="1">
       <c r="A116" s="5" t="inlineStr">
         <is>
-          <t>19:10-19:20</t>
+          <t>19:00-19:10</t>
         </is>
       </c>
       <c r="B116" s="7" t="n">
@@ -1620,7 +1620,7 @@
     <row r="117" ht="14" customHeight="1">
       <c r="A117" s="5" t="inlineStr">
         <is>
-          <t>19:20-19:30</t>
+          <t>19:10-19:20</t>
         </is>
       </c>
       <c r="B117" s="7" t="n">
@@ -1630,7 +1630,7 @@
     <row r="118" ht="14" customHeight="1">
       <c r="A118" s="5" t="inlineStr">
         <is>
-          <t>19:30-19:40</t>
+          <t>19:20-19:30</t>
         </is>
       </c>
       <c r="B118" s="7" t="n">
@@ -1640,7 +1640,7 @@
     <row r="119" ht="14" customHeight="1">
       <c r="A119" s="5" t="inlineStr">
         <is>
-          <t>19:40-19:50</t>
+          <t>19:30-19:40</t>
         </is>
       </c>
       <c r="B119" s="7" t="n">
@@ -1650,7 +1650,7 @@
     <row r="120" ht="14" customHeight="1">
       <c r="A120" s="5" t="inlineStr">
         <is>
-          <t>19:50-20:00</t>
+          <t>19:40-19:50</t>
         </is>
       </c>
       <c r="B120" s="7" t="n">
@@ -1660,7 +1660,7 @@
     <row r="121" ht="14" customHeight="1">
       <c r="A121" s="5" t="inlineStr">
         <is>
-          <t>20:00-20:10</t>
+          <t>19:50-20:00</t>
         </is>
       </c>
       <c r="B121" s="7" t="n">
@@ -1670,7 +1670,7 @@
     <row r="122" ht="14" customHeight="1">
       <c r="A122" s="5" t="inlineStr">
         <is>
-          <t>20:10-20:20</t>
+          <t>20:00-20:10</t>
         </is>
       </c>
       <c r="B122" s="7" t="n">
@@ -1680,7 +1680,7 @@
     <row r="123" ht="14" customHeight="1">
       <c r="A123" s="5" t="inlineStr">
         <is>
-          <t>20:20-20:30</t>
+          <t>20:10-20:20</t>
         </is>
       </c>
       <c r="B123" s="7" t="n">
@@ -1690,7 +1690,7 @@
     <row r="124" ht="14" customHeight="1">
       <c r="A124" s="5" t="inlineStr">
         <is>
-          <t>20:30-20:40</t>
+          <t>20:20-20:30</t>
         </is>
       </c>
       <c r="B124" s="7" t="n">
@@ -1700,7 +1700,7 @@
     <row r="125" ht="14" customHeight="1">
       <c r="A125" s="5" t="inlineStr">
         <is>
-          <t>20:40-20:50</t>
+          <t>20:30-20:40</t>
         </is>
       </c>
       <c r="B125" s="7" t="n">
@@ -1710,7 +1710,7 @@
     <row r="126" ht="14" customHeight="1">
       <c r="A126" s="5" t="inlineStr">
         <is>
-          <t>20:50-21:00</t>
+          <t>20:40-20:50</t>
         </is>
       </c>
       <c r="B126" s="7" t="n">
@@ -1720,7 +1720,7 @@
     <row r="127" ht="14" customHeight="1">
       <c r="A127" s="5" t="inlineStr">
         <is>
-          <t>21:00-21:10</t>
+          <t>20:50-21:00</t>
         </is>
       </c>
       <c r="B127" s="7" t="n">
@@ -1730,7 +1730,7 @@
     <row r="128" ht="14" customHeight="1">
       <c r="A128" s="5" t="inlineStr">
         <is>
-          <t>21:10-21:20</t>
+          <t>21:00-21:10</t>
         </is>
       </c>
       <c r="B128" s="7" t="n">
@@ -1740,7 +1740,7 @@
     <row r="129" ht="14" customHeight="1">
       <c r="A129" s="5" t="inlineStr">
         <is>
-          <t>21:20-21:30</t>
+          <t>21:10-21:20</t>
         </is>
       </c>
       <c r="B129" s="7" t="n">
@@ -1750,7 +1750,7 @@
     <row r="130" ht="14" customHeight="1">
       <c r="A130" s="5" t="inlineStr">
         <is>
-          <t>21:30-21:40</t>
+          <t>21:20-21:30</t>
         </is>
       </c>
       <c r="B130" s="7" t="n">
@@ -1760,7 +1760,7 @@
     <row r="131" ht="14" customHeight="1">
       <c r="A131" s="5" t="inlineStr">
         <is>
-          <t>21:40-21:50</t>
+          <t>21:30-21:40</t>
         </is>
       </c>
       <c r="B131" s="7" t="n">
@@ -1770,7 +1770,7 @@
     <row r="132" ht="14" customHeight="1">
       <c r="A132" s="5" t="inlineStr">
         <is>
-          <t>21:50-22:00</t>
+          <t>21:40-21:50</t>
         </is>
       </c>
       <c r="B132" s="7" t="n">
@@ -1780,27 +1780,27 @@
     <row r="133" ht="14" customHeight="1">
       <c r="A133" s="5" t="inlineStr">
         <is>
-          <t>22:00-22:10</t>
+          <t>21:50-22:00</t>
         </is>
       </c>
       <c r="B133" s="7" t="n">
-        <v>1486.3829</v>
+        <v>1393.7903</v>
       </c>
     </row>
     <row r="134" ht="14" customHeight="1">
       <c r="A134" s="5" t="inlineStr">
         <is>
-          <t>22:10-22:20</t>
+          <t>22:00-22:10</t>
         </is>
       </c>
       <c r="B134" s="7" t="n">
-        <v>1477.4915</v>
+        <v>1384.8989</v>
       </c>
     </row>
     <row r="135" ht="14" customHeight="1">
       <c r="A135" s="5" t="inlineStr">
         <is>
-          <t>22:20-22:30</t>
+          <t>22:10-22:20</t>
         </is>
       </c>
       <c r="B135" s="7" t="n">
@@ -1810,27 +1810,27 @@
     <row r="136" ht="14" customHeight="1">
       <c r="A136" s="5" t="inlineStr">
         <is>
-          <t>22:30-22:40</t>
+          <t>22:20-22:30</t>
         </is>
       </c>
       <c r="B136" s="7" t="n">
-        <v>1489.5811</v>
+        <v>1396.9885</v>
       </c>
     </row>
     <row r="137" ht="14" customHeight="1">
       <c r="A137" s="5" t="inlineStr">
         <is>
-          <t>22:40-22:50</t>
+          <t>22:30-22:40</t>
         </is>
       </c>
       <c r="B137" s="7" t="n">
-        <v>1490.3525</v>
+        <v>1397.7599</v>
       </c>
     </row>
     <row r="138" ht="14" customHeight="1">
       <c r="A138" s="5" t="inlineStr">
         <is>
-          <t>22:50-23:00</t>
+          <t>22:40-22:50</t>
         </is>
       </c>
       <c r="B138" s="7" t="n">
@@ -1840,17 +1840,17 @@
     <row r="139" ht="14" customHeight="1">
       <c r="A139" s="5" t="inlineStr">
         <is>
-          <t>23:00-23:10</t>
+          <t>22:50-23:00</t>
         </is>
       </c>
       <c r="B139" s="7" t="n">
-        <v>1270.2441</v>
+        <v>1399.8738</v>
       </c>
     </row>
     <row r="140" ht="14" customHeight="1">
       <c r="A140" s="5" t="inlineStr">
         <is>
-          <t>23:10-23:20</t>
+          <t>23:00-23:10</t>
         </is>
       </c>
       <c r="B140" s="7" t="n">
@@ -1860,7 +1860,7 @@
     <row r="141" ht="14" customHeight="1">
       <c r="A141" s="5" t="inlineStr">
         <is>
-          <t>23:20-23:30</t>
+          <t>23:10-23:20</t>
         </is>
       </c>
       <c r="B141" s="7" t="n">
@@ -1870,27 +1870,27 @@
     <row r="142" ht="14" customHeight="1">
       <c r="A142" s="5" t="inlineStr">
         <is>
-          <t>23:30-23:40</t>
+          <t>23:20-23:30</t>
         </is>
       </c>
       <c r="B142" s="7" t="n">
-        <v>1496.2561</v>
+        <v>1403.6635</v>
       </c>
     </row>
     <row r="143" ht="14" customHeight="1">
       <c r="A143" s="5" t="inlineStr">
         <is>
-          <t>23:40-23:50</t>
+          <t>23:30-23:40</t>
         </is>
       </c>
       <c r="B143" s="7" t="n">
-        <v>571.61538</v>
+        <v>904.94872</v>
       </c>
     </row>
     <row r="144" ht="14" customHeight="1">
       <c r="A144" s="5" t="inlineStr">
         <is>
-          <t>23:50-0:00+1</t>
+          <t>23:40-23:50</t>
         </is>
       </c>
       <c r="B144" s="7" t="n">
@@ -1900,7 +1900,7 @@
     <row r="145" ht="14" customHeight="1">
       <c r="A145" s="5" t="inlineStr">
         <is>
-          <t>0:00+1-0:10+1</t>
+          <t>23:50-24:00</t>
         </is>
       </c>
       <c r="B145" s="7" t="n">
@@ -1960,7 +1960,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>3966.66665</v>
+        <v>4050</v>
       </c>
       <c r="C2" t="n">
         <v>0</v>
@@ -1981,7 +1981,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>833.33333</v>
+        <v>750</v>
       </c>
       <c r="C3" t="n">
         <v>7073.15689</v>
@@ -2002,7 +2002,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>3975.834515</v>
+        <v>4309.167855</v>
       </c>
       <c r="C4" t="n">
         <v>1892.218881</v>
@@ -2015,7 +2015,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>5090.764985</v>
+        <v>4757.431665</v>
       </c>
       <c r="C5" t="n">
         <v>101.22376</v>
@@ -2041,7 +2041,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>4799.999980000001</v>
+        <v>4800</v>
       </c>
       <c r="C7" t="n">
         <v>3177.63125</v>

</xml_diff>

<commit_message>
results(Q1): rerun after start-align
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/results/Q1/result1.xlsx
+++ b/results/Q1/result1.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-110" yWindow="-110" windowWidth="25420" windowHeight="16300" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="计划购电量" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="充放电量" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="计划购电量" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="充放电量" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -470,7 +470,7 @@
     <row r="2" ht="14" customHeight="1">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>00:00-00:10</t>
+          <t>0:10-0:20</t>
         </is>
       </c>
       <c r="B2" s="7" t="n">
@@ -480,7 +480,7 @@
     <row r="3" ht="14" customHeight="1">
       <c r="A3" s="5" t="inlineStr">
         <is>
-          <t>00:10-00:20</t>
+          <t>0:20-0:30</t>
         </is>
       </c>
       <c r="B3" s="7" t="n">
@@ -490,7 +490,7 @@
     <row r="4" ht="14" customHeight="1">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>00:20-00:30</t>
+          <t>0:30-0:40</t>
         </is>
       </c>
       <c r="B4" s="7" t="n">
@@ -500,7 +500,7 @@
     <row r="5" ht="14" customHeight="1">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>00:30-00:40</t>
+          <t>0:40-0:50</t>
         </is>
       </c>
       <c r="B5" s="7" t="n">
@@ -510,7 +510,7 @@
     <row r="6" ht="14" customHeight="1">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>00:40-00:50</t>
+          <t>0:50-1:00</t>
         </is>
       </c>
       <c r="B6" s="7" t="n">
@@ -520,7 +520,7 @@
     <row r="7" ht="14" customHeight="1">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>00:50-01:00</t>
+          <t>1:00-1:10</t>
         </is>
       </c>
       <c r="B7" s="7" t="n">
@@ -530,7 +530,7 @@
     <row r="8" ht="14" customHeight="1">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>01:00-01:10</t>
+          <t>1:10-1:20</t>
         </is>
       </c>
       <c r="B8" s="7" t="n">
@@ -540,7 +540,7 @@
     <row r="9" ht="14" customHeight="1">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>01:10-01:20</t>
+          <t>1:20-1:30</t>
         </is>
       </c>
       <c r="B9" s="7" t="n">
@@ -550,17 +550,17 @@
     <row r="10" ht="14" customHeight="1">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>01:20-01:30</t>
+          <t>1:30-1:40</t>
         </is>
       </c>
       <c r="B10" s="7" t="n">
-        <v>911.16138</v>
+        <v>577.82805</v>
       </c>
     </row>
     <row r="11" ht="14" customHeight="1">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>01:30-01:40</t>
+          <t>1:40-1:50</t>
         </is>
       </c>
       <c r="B11" s="7" t="n">
@@ -570,7 +570,7 @@
     <row r="12" ht="14" customHeight="1">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>01:40-01:50</t>
+          <t>1:50-2:00</t>
         </is>
       </c>
       <c r="B12" s="7" t="n">
@@ -580,7 +580,7 @@
     <row r="13" ht="14" customHeight="1">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>01:50-02:00</t>
+          <t>2:00-2:10</t>
         </is>
       </c>
       <c r="B13" s="7" t="n">
@@ -590,7 +590,7 @@
     <row r="14" ht="14" customHeight="1">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>02:00-02:10</t>
+          <t>2:10-2:20</t>
         </is>
       </c>
       <c r="B14" s="7" t="n">
@@ -600,7 +600,7 @@
     <row r="15" ht="14" customHeight="1">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>02:10-02:20</t>
+          <t>2:20-2:30</t>
         </is>
       </c>
       <c r="B15" s="7" t="n">
@@ -610,7 +610,7 @@
     <row r="16" ht="14" customHeight="1">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>02:20-02:30</t>
+          <t>2:30-2:40</t>
         </is>
       </c>
       <c r="B16" s="7" t="n">
@@ -620,7 +620,7 @@
     <row r="17" ht="14" customHeight="1">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>02:30-02:40</t>
+          <t>2:40-2:50</t>
         </is>
       </c>
       <c r="B17" s="7" t="n">
@@ -630,7 +630,7 @@
     <row r="18" ht="14" customHeight="1">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>02:40-02:50</t>
+          <t>2:50-3:00</t>
         </is>
       </c>
       <c r="B18" s="7" t="n">
@@ -640,7 +640,7 @@
     <row r="19" ht="14" customHeight="1">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>02:50-03:00</t>
+          <t>3:00-3:10</t>
         </is>
       </c>
       <c r="B19" s="7" t="n">
@@ -650,7 +650,7 @@
     <row r="20" ht="14" customHeight="1">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t>03:00-03:10</t>
+          <t>3:10-3:20</t>
         </is>
       </c>
       <c r="B20" s="7" t="n">
@@ -660,7 +660,7 @@
     <row r="21" ht="14" customHeight="1">
       <c r="A21" s="5" t="inlineStr">
         <is>
-          <t>03:10-03:20</t>
+          <t>3:20-3:30</t>
         </is>
       </c>
       <c r="B21" s="7" t="n">
@@ -670,7 +670,7 @@
     <row r="22" ht="14" customHeight="1">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>03:20-03:30</t>
+          <t>3:30-3:40</t>
         </is>
       </c>
       <c r="B22" s="7" t="n">
@@ -680,7 +680,7 @@
     <row r="23" ht="14" customHeight="1">
       <c r="A23" s="5" t="inlineStr">
         <is>
-          <t>03:30-03:40</t>
+          <t>3:40-3:50</t>
         </is>
       </c>
       <c r="B23" s="7" t="n">
@@ -690,7 +690,7 @@
     <row r="24" ht="14" customHeight="1">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>03:40-03:50</t>
+          <t>3:50-4:00</t>
         </is>
       </c>
       <c r="B24" s="7" t="n">
@@ -700,7 +700,7 @@
     <row r="25" ht="14" customHeight="1">
       <c r="A25" s="5" t="inlineStr">
         <is>
-          <t>03:50-04:00</t>
+          <t>4:00-4:10</t>
         </is>
       </c>
       <c r="B25" s="7" t="n">
@@ -710,7 +710,7 @@
     <row r="26" ht="14" customHeight="1">
       <c r="A26" s="5" t="inlineStr">
         <is>
-          <t>04:00-04:10</t>
+          <t>4:10-4:20</t>
         </is>
       </c>
       <c r="B26" s="7" t="n">
@@ -720,7 +720,7 @@
     <row r="27" ht="14" customHeight="1">
       <c r="A27" s="5" t="inlineStr">
         <is>
-          <t>04:10-04:20</t>
+          <t>4:20-4:30</t>
         </is>
       </c>
       <c r="B27" s="7" t="n">
@@ -730,7 +730,7 @@
     <row r="28" ht="14" customHeight="1">
       <c r="A28" s="5" t="inlineStr">
         <is>
-          <t>04:20-04:30</t>
+          <t>4:30-4:40</t>
         </is>
       </c>
       <c r="B28" s="7" t="n">
@@ -740,7 +740,7 @@
     <row r="29" ht="14" customHeight="1">
       <c r="A29" s="5" t="inlineStr">
         <is>
-          <t>04:30-04:40</t>
+          <t>4:40-4:50</t>
         </is>
       </c>
       <c r="B29" s="7" t="n">
@@ -750,7 +750,7 @@
     <row r="30" ht="14" customHeight="1">
       <c r="A30" s="5" t="inlineStr">
         <is>
-          <t>04:40-04:50</t>
+          <t>4:50-5:00</t>
         </is>
       </c>
       <c r="B30" s="7" t="n">
@@ -760,7 +760,7 @@
     <row r="31" ht="14" customHeight="1">
       <c r="A31" s="5" t="inlineStr">
         <is>
-          <t>04:50-05:00</t>
+          <t>5:00-5:10</t>
         </is>
       </c>
       <c r="B31" s="7" t="n">
@@ -770,7 +770,7 @@
     <row r="32" ht="14" customHeight="1">
       <c r="A32" s="5" t="inlineStr">
         <is>
-          <t>05:00-05:10</t>
+          <t>5:10-5:20</t>
         </is>
       </c>
       <c r="B32" s="7" t="n">
@@ -780,7 +780,7 @@
     <row r="33" ht="14" customHeight="1">
       <c r="A33" s="5" t="inlineStr">
         <is>
-          <t>05:10-05:20</t>
+          <t>5:20-5:30</t>
         </is>
       </c>
       <c r="B33" s="7" t="n">
@@ -790,7 +790,7 @@
     <row r="34" ht="14" customHeight="1">
       <c r="A34" s="5" t="inlineStr">
         <is>
-          <t>05:20-05:30</t>
+          <t>5:30-5:40</t>
         </is>
       </c>
       <c r="B34" s="7" t="n">
@@ -800,7 +800,7 @@
     <row r="35" ht="14" customHeight="1">
       <c r="A35" s="5" t="inlineStr">
         <is>
-          <t>05:30-05:40</t>
+          <t>5:40-5:50</t>
         </is>
       </c>
       <c r="B35" s="7" t="n">
@@ -810,7 +810,7 @@
     <row r="36" ht="14" customHeight="1">
       <c r="A36" s="5" t="inlineStr">
         <is>
-          <t>05:40-05:50</t>
+          <t>5:50-6:00</t>
         </is>
       </c>
       <c r="B36" s="7" t="n">
@@ -820,7 +820,7 @@
     <row r="37" ht="14" customHeight="1">
       <c r="A37" s="5" t="inlineStr">
         <is>
-          <t>05:50-06:00</t>
+          <t>6:00-6:10</t>
         </is>
       </c>
       <c r="B37" s="7" t="n">
@@ -830,7 +830,7 @@
     <row r="38" ht="14" customHeight="1">
       <c r="A38" s="5" t="inlineStr">
         <is>
-          <t>06:00-06:10</t>
+          <t>6:10-6:20</t>
         </is>
       </c>
       <c r="B38" s="7" t="n">
@@ -840,7 +840,7 @@
     <row r="39" ht="14" customHeight="1">
       <c r="A39" s="5" t="inlineStr">
         <is>
-          <t>06:10-06:20</t>
+          <t>6:20-6:30</t>
         </is>
       </c>
       <c r="B39" s="7" t="n">
@@ -850,7 +850,7 @@
     <row r="40" ht="14" customHeight="1">
       <c r="A40" s="5" t="inlineStr">
         <is>
-          <t>06:20-06:30</t>
+          <t>6:30-6:40</t>
         </is>
       </c>
       <c r="B40" s="7" t="n">
@@ -860,7 +860,7 @@
     <row r="41" ht="14" customHeight="1">
       <c r="A41" s="5" t="inlineStr">
         <is>
-          <t>06:30-06:40</t>
+          <t>6:40-6:50</t>
         </is>
       </c>
       <c r="B41" s="7" t="n">
@@ -870,7 +870,7 @@
     <row r="42" ht="14" customHeight="1">
       <c r="A42" s="5" t="inlineStr">
         <is>
-          <t>06:40-06:50</t>
+          <t>6:50-7:00</t>
         </is>
       </c>
       <c r="B42" s="7" t="n">
@@ -880,7 +880,7 @@
     <row r="43" ht="14" customHeight="1">
       <c r="A43" s="5" t="inlineStr">
         <is>
-          <t>06:50-07:00</t>
+          <t>7:00-7:10</t>
         </is>
       </c>
       <c r="B43" s="7" t="n">
@@ -890,7 +890,7 @@
     <row r="44" ht="14" customHeight="1">
       <c r="A44" s="5" t="inlineStr">
         <is>
-          <t>07:00-07:10</t>
+          <t>7:10-7:20</t>
         </is>
       </c>
       <c r="B44" s="7" t="n">
@@ -900,7 +900,7 @@
     <row r="45" ht="14" customHeight="1">
       <c r="A45" s="5" t="inlineStr">
         <is>
-          <t>07:10-07:20</t>
+          <t>7:20-7:30</t>
         </is>
       </c>
       <c r="B45" s="7" t="n">
@@ -910,7 +910,7 @@
     <row r="46" ht="14" customHeight="1">
       <c r="A46" s="5" t="inlineStr">
         <is>
-          <t>07:20-07:30</t>
+          <t>7:30-7:40</t>
         </is>
       </c>
       <c r="B46" s="7" t="n">
@@ -920,7 +920,7 @@
     <row r="47" ht="14" customHeight="1">
       <c r="A47" s="5" t="inlineStr">
         <is>
-          <t>07:30-07:40</t>
+          <t>7:40-7:50</t>
         </is>
       </c>
       <c r="B47" s="7" t="n">
@@ -930,7 +930,7 @@
     <row r="48" ht="14" customHeight="1">
       <c r="A48" s="5" t="inlineStr">
         <is>
-          <t>07:40-07:50</t>
+          <t>7:50-8:00</t>
         </is>
       </c>
       <c r="B48" s="7" t="n">
@@ -940,7 +940,7 @@
     <row r="49" ht="14" customHeight="1">
       <c r="A49" s="5" t="inlineStr">
         <is>
-          <t>07:50-08:00</t>
+          <t>8:00-8:10</t>
         </is>
       </c>
       <c r="B49" s="7" t="n">
@@ -950,7 +950,7 @@
     <row r="50" ht="14" customHeight="1">
       <c r="A50" s="5" t="inlineStr">
         <is>
-          <t>08:00-08:10</t>
+          <t>8:10-8:20</t>
         </is>
       </c>
       <c r="B50" s="7" t="n">
@@ -960,7 +960,7 @@
     <row r="51" ht="14" customHeight="1">
       <c r="A51" s="5" t="inlineStr">
         <is>
-          <t>08:10-08:20</t>
+          <t>8:20-8:30</t>
         </is>
       </c>
       <c r="B51" s="7" t="n">
@@ -970,7 +970,7 @@
     <row r="52" ht="14" customHeight="1">
       <c r="A52" s="5" t="inlineStr">
         <is>
-          <t>08:20-08:30</t>
+          <t>8:30-8:40</t>
         </is>
       </c>
       <c r="B52" s="7" t="n">
@@ -980,7 +980,7 @@
     <row r="53" ht="14" customHeight="1">
       <c r="A53" s="5" t="inlineStr">
         <is>
-          <t>08:30-08:40</t>
+          <t>8:40-8:50</t>
         </is>
       </c>
       <c r="B53" s="7" t="n">
@@ -990,7 +990,7 @@
     <row r="54" ht="14" customHeight="1">
       <c r="A54" s="5" t="inlineStr">
         <is>
-          <t>08:40-08:50</t>
+          <t>8:50-9:00</t>
         </is>
       </c>
       <c r="B54" s="7" t="n">
@@ -1000,7 +1000,7 @@
     <row r="55" ht="14" customHeight="1">
       <c r="A55" s="5" t="inlineStr">
         <is>
-          <t>08:50-09:00</t>
+          <t>9:00-9:10</t>
         </is>
       </c>
       <c r="B55" s="7" t="n">
@@ -1010,7 +1010,7 @@
     <row r="56" ht="14" customHeight="1">
       <c r="A56" s="5" t="inlineStr">
         <is>
-          <t>09:00-09:10</t>
+          <t>9:10-9:20</t>
         </is>
       </c>
       <c r="B56" s="7" t="n">
@@ -1020,7 +1020,7 @@
     <row r="57" ht="14" customHeight="1">
       <c r="A57" s="5" t="inlineStr">
         <is>
-          <t>09:10-09:20</t>
+          <t>9:20-9:30</t>
         </is>
       </c>
       <c r="B57" s="7" t="n">
@@ -1030,7 +1030,7 @@
     <row r="58" ht="14" customHeight="1">
       <c r="A58" s="5" t="inlineStr">
         <is>
-          <t>09:20-09:30</t>
+          <t>9:30-9:40</t>
         </is>
       </c>
       <c r="B58" s="7" t="n">
@@ -1040,7 +1040,7 @@
     <row r="59" ht="14" customHeight="1">
       <c r="A59" s="5" t="inlineStr">
         <is>
-          <t>09:30-09:40</t>
+          <t>9:40-9:50</t>
         </is>
       </c>
       <c r="B59" s="7" t="n">
@@ -1050,7 +1050,7 @@
     <row r="60" ht="14" customHeight="1">
       <c r="A60" s="5" t="inlineStr">
         <is>
-          <t>09:40-09:50</t>
+          <t>9:50-10:00</t>
         </is>
       </c>
       <c r="B60" s="7" t="n">
@@ -1060,7 +1060,7 @@
     <row r="61" ht="14" customHeight="1">
       <c r="A61" s="5" t="inlineStr">
         <is>
-          <t>09:50-10:00</t>
+          <t>10:00-10:10</t>
         </is>
       </c>
       <c r="B61" s="7" t="n">
@@ -1070,7 +1070,7 @@
     <row r="62" ht="14" customHeight="1">
       <c r="A62" s="5" t="inlineStr">
         <is>
-          <t>10:00-10:10</t>
+          <t>10:10-10:20</t>
         </is>
       </c>
       <c r="B62" s="7" t="n">
@@ -1080,7 +1080,7 @@
     <row r="63" ht="14" customHeight="1">
       <c r="A63" s="5" t="inlineStr">
         <is>
-          <t>10:10-10:20</t>
+          <t>10:20-10:30</t>
         </is>
       </c>
       <c r="B63" s="7" t="n">
@@ -1090,7 +1090,7 @@
     <row r="64" ht="14" customHeight="1">
       <c r="A64" s="5" t="inlineStr">
         <is>
-          <t>10:20-10:30</t>
+          <t>10:30-10:40</t>
         </is>
       </c>
       <c r="B64" s="7" t="n">
@@ -1100,7 +1100,7 @@
     <row r="65" ht="14" customHeight="1">
       <c r="A65" s="5" t="inlineStr">
         <is>
-          <t>10:30-10:40</t>
+          <t>10:40-10:50</t>
         </is>
       </c>
       <c r="B65" s="7" t="n">
@@ -1110,7 +1110,7 @@
     <row r="66" ht="14" customHeight="1">
       <c r="A66" s="5" t="inlineStr">
         <is>
-          <t>10:40-10:50</t>
+          <t>10:50-11:00</t>
         </is>
       </c>
       <c r="B66" s="7" t="n">
@@ -1120,7 +1120,7 @@
     <row r="67" ht="14" customHeight="1">
       <c r="A67" s="5" t="inlineStr">
         <is>
-          <t>10:50-11:00</t>
+          <t>11:00-11:10</t>
         </is>
       </c>
       <c r="B67" s="7" t="n">
@@ -1130,7 +1130,7 @@
     <row r="68" ht="14" customHeight="1">
       <c r="A68" s="5" t="inlineStr">
         <is>
-          <t>11:00-11:10</t>
+          <t>11:10-11:20</t>
         </is>
       </c>
       <c r="B68" s="7" t="n">
@@ -1140,7 +1140,7 @@
     <row r="69" ht="14" customHeight="1">
       <c r="A69" s="5" t="inlineStr">
         <is>
-          <t>11:10-11:20</t>
+          <t>11:20-11:30</t>
         </is>
       </c>
       <c r="B69" s="7" t="n">
@@ -1150,7 +1150,7 @@
     <row r="70" ht="14" customHeight="1">
       <c r="A70" s="5" t="inlineStr">
         <is>
-          <t>11:20-11:30</t>
+          <t>11:30-11:40</t>
         </is>
       </c>
       <c r="B70" s="7" t="n">
@@ -1160,7 +1160,7 @@
     <row r="71" ht="14" customHeight="1">
       <c r="A71" s="5" t="inlineStr">
         <is>
-          <t>11:30-11:40</t>
+          <t>11:40-11:50</t>
         </is>
       </c>
       <c r="B71" s="7" t="n">
@@ -1170,7 +1170,7 @@
     <row r="72" ht="14" customHeight="1">
       <c r="A72" s="5" t="inlineStr">
         <is>
-          <t>11:40-11:50</t>
+          <t>11:50-12:00</t>
         </is>
       </c>
       <c r="B72" s="7" t="n">
@@ -1180,7 +1180,7 @@
     <row r="73" ht="14" customHeight="1">
       <c r="A73" s="5" t="inlineStr">
         <is>
-          <t>11:50-12:00</t>
+          <t>12:00-12:10</t>
         </is>
       </c>
       <c r="B73" s="7" t="n">
@@ -1190,7 +1190,7 @@
     <row r="74" ht="14" customHeight="1">
       <c r="A74" s="5" t="inlineStr">
         <is>
-          <t>12:00-12:10</t>
+          <t>12:10-12:20</t>
         </is>
       </c>
       <c r="B74" s="7" t="n">
@@ -1200,7 +1200,7 @@
     <row r="75" ht="14" customHeight="1">
       <c r="A75" s="5" t="inlineStr">
         <is>
-          <t>12:10-12:20</t>
+          <t>12:20-12:30</t>
         </is>
       </c>
       <c r="B75" s="7" t="n">
@@ -1210,7 +1210,7 @@
     <row r="76" ht="14" customHeight="1">
       <c r="A76" s="5" t="inlineStr">
         <is>
-          <t>12:20-12:30</t>
+          <t>12:30-12:40</t>
         </is>
       </c>
       <c r="B76" s="7" t="n">
@@ -1220,7 +1220,7 @@
     <row r="77" ht="14" customHeight="1">
       <c r="A77" s="5" t="inlineStr">
         <is>
-          <t>12:30-12:40</t>
+          <t>12:40-12:50</t>
         </is>
       </c>
       <c r="B77" s="7" t="n">
@@ -1230,7 +1230,7 @@
     <row r="78" ht="14" customHeight="1">
       <c r="A78" s="5" t="inlineStr">
         <is>
-          <t>12:40-12:50</t>
+          <t>12:50-13:00</t>
         </is>
       </c>
       <c r="B78" s="7" t="n">
@@ -1240,7 +1240,7 @@
     <row r="79" ht="14" customHeight="1">
       <c r="A79" s="5" t="inlineStr">
         <is>
-          <t>12:50-13:00</t>
+          <t>13:00-13:10</t>
         </is>
       </c>
       <c r="B79" s="7" t="n">
@@ -1250,7 +1250,7 @@
     <row r="80" ht="14" customHeight="1">
       <c r="A80" s="5" t="inlineStr">
         <is>
-          <t>13:00-13:10</t>
+          <t>13:10-13:20</t>
         </is>
       </c>
       <c r="B80" s="7" t="n">
@@ -1260,7 +1260,7 @@
     <row r="81" ht="14" customHeight="1">
       <c r="A81" s="5" t="inlineStr">
         <is>
-          <t>13:10-13:20</t>
+          <t>13:20-13:30</t>
         </is>
       </c>
       <c r="B81" s="7" t="n">
@@ -1270,7 +1270,7 @@
     <row r="82" ht="14" customHeight="1">
       <c r="A82" s="5" t="inlineStr">
         <is>
-          <t>13:20-13:30</t>
+          <t>13:30-13:40</t>
         </is>
       </c>
       <c r="B82" s="7" t="n">
@@ -1280,7 +1280,7 @@
     <row r="83" ht="14" customHeight="1">
       <c r="A83" s="5" t="inlineStr">
         <is>
-          <t>13:30-13:40</t>
+          <t>13:40-13:50</t>
         </is>
       </c>
       <c r="B83" s="7" t="n">
@@ -1290,7 +1290,7 @@
     <row r="84" ht="14" customHeight="1">
       <c r="A84" s="5" t="inlineStr">
         <is>
-          <t>13:40-13:50</t>
+          <t>13:50-14:00</t>
         </is>
       </c>
       <c r="B84" s="7" t="n">
@@ -1300,7 +1300,7 @@
     <row r="85" ht="14" customHeight="1">
       <c r="A85" s="5" t="inlineStr">
         <is>
-          <t>13:50-14:00</t>
+          <t>14:00-14:10</t>
         </is>
       </c>
       <c r="B85" s="7" t="n">
@@ -1310,7 +1310,7 @@
     <row r="86" ht="14" customHeight="1">
       <c r="A86" s="5" t="inlineStr">
         <is>
-          <t>14:00-14:10</t>
+          <t>14:10-14:20</t>
         </is>
       </c>
       <c r="B86" s="7" t="n">
@@ -1320,7 +1320,7 @@
     <row r="87" ht="14" customHeight="1">
       <c r="A87" s="5" t="inlineStr">
         <is>
-          <t>14:10-14:20</t>
+          <t>14:20-14:30</t>
         </is>
       </c>
       <c r="B87" s="7" t="n">
@@ -1330,7 +1330,7 @@
     <row r="88" ht="14" customHeight="1">
       <c r="A88" s="5" t="inlineStr">
         <is>
-          <t>14:20-14:30</t>
+          <t>14:30-14:40</t>
         </is>
       </c>
       <c r="B88" s="7" t="n">
@@ -1340,7 +1340,7 @@
     <row r="89" ht="14" customHeight="1">
       <c r="A89" s="5" t="inlineStr">
         <is>
-          <t>14:30-14:40</t>
+          <t>14:40-14:50</t>
         </is>
       </c>
       <c r="B89" s="7" t="n">
@@ -1350,7 +1350,7 @@
     <row r="90" ht="14" customHeight="1">
       <c r="A90" s="5" t="inlineStr">
         <is>
-          <t>14:40-14:50</t>
+          <t>14:50-15:00</t>
         </is>
       </c>
       <c r="B90" s="7" t="n">
@@ -1360,7 +1360,7 @@
     <row r="91" ht="14" customHeight="1">
       <c r="A91" s="5" t="inlineStr">
         <is>
-          <t>14:50-15:00</t>
+          <t>15:00-15:10</t>
         </is>
       </c>
       <c r="B91" s="7" t="n">
@@ -1370,7 +1370,7 @@
     <row r="92" ht="14" customHeight="1">
       <c r="A92" s="5" t="inlineStr">
         <is>
-          <t>15:00-15:10</t>
+          <t>15:10-15:20</t>
         </is>
       </c>
       <c r="B92" s="7" t="n">
@@ -1380,7 +1380,7 @@
     <row r="93" ht="14" customHeight="1">
       <c r="A93" s="5" t="inlineStr">
         <is>
-          <t>15:10-15:20</t>
+          <t>15:20-15:30</t>
         </is>
       </c>
       <c r="B93" s="7" t="n">
@@ -1390,7 +1390,7 @@
     <row r="94" ht="14" customHeight="1">
       <c r="A94" s="5" t="inlineStr">
         <is>
-          <t>15:20-15:30</t>
+          <t>15:30-15:40</t>
         </is>
       </c>
       <c r="B94" s="7" t="n">
@@ -1400,7 +1400,7 @@
     <row r="95" ht="14" customHeight="1">
       <c r="A95" s="5" t="inlineStr">
         <is>
-          <t>15:30-15:40</t>
+          <t>15:40-15:50</t>
         </is>
       </c>
       <c r="B95" s="7" t="n">
@@ -1410,7 +1410,7 @@
     <row r="96" ht="14" customHeight="1">
       <c r="A96" s="5" t="inlineStr">
         <is>
-          <t>15:40-15:50</t>
+          <t>15:50-16:00</t>
         </is>
       </c>
       <c r="B96" s="7" t="n">
@@ -1420,7 +1420,7 @@
     <row r="97" ht="14" customHeight="1">
       <c r="A97" s="5" t="inlineStr">
         <is>
-          <t>15:50-16:00</t>
+          <t>16:00-16:10</t>
         </is>
       </c>
       <c r="B97" s="7" t="n">
@@ -1430,7 +1430,7 @@
     <row r="98" ht="14" customHeight="1">
       <c r="A98" s="5" t="inlineStr">
         <is>
-          <t>16:00-16:10</t>
+          <t>16:10-16:20</t>
         </is>
       </c>
       <c r="B98" s="7" t="n">
@@ -1440,7 +1440,7 @@
     <row r="99" ht="14" customHeight="1">
       <c r="A99" s="5" t="inlineStr">
         <is>
-          <t>16:10-16:20</t>
+          <t>16:20-16:30</t>
         </is>
       </c>
       <c r="B99" s="7" t="n">
@@ -1450,7 +1450,7 @@
     <row r="100" ht="14" customHeight="1">
       <c r="A100" s="5" t="inlineStr">
         <is>
-          <t>16:20-16:30</t>
+          <t>16:30-16:40</t>
         </is>
       </c>
       <c r="B100" s="7" t="n">
@@ -1460,7 +1460,7 @@
     <row r="101" ht="14" customHeight="1">
       <c r="A101" s="5" t="inlineStr">
         <is>
-          <t>16:30-16:40</t>
+          <t>16:40-16:50</t>
         </is>
       </c>
       <c r="B101" s="7" t="n">
@@ -1470,7 +1470,7 @@
     <row r="102" ht="14" customHeight="1">
       <c r="A102" s="5" t="inlineStr">
         <is>
-          <t>16:40-16:50</t>
+          <t>16:50-17:00</t>
         </is>
       </c>
       <c r="B102" s="7" t="n">
@@ -1480,7 +1480,7 @@
     <row r="103" ht="14" customHeight="1">
       <c r="A103" s="5" t="inlineStr">
         <is>
-          <t>16:50-17:00</t>
+          <t>17:00-17:10</t>
         </is>
       </c>
       <c r="B103" s="7" t="n">
@@ -1490,7 +1490,7 @@
     <row r="104" ht="14" customHeight="1">
       <c r="A104" s="5" t="inlineStr">
         <is>
-          <t>17:00-17:10</t>
+          <t>17:10-17:20</t>
         </is>
       </c>
       <c r="B104" s="7" t="n">
@@ -1500,7 +1500,7 @@
     <row r="105" ht="14" customHeight="1">
       <c r="A105" s="5" t="inlineStr">
         <is>
-          <t>17:10-17:20</t>
+          <t>17:20-17:30</t>
         </is>
       </c>
       <c r="B105" s="7" t="n">
@@ -1510,7 +1510,7 @@
     <row r="106" ht="14" customHeight="1">
       <c r="A106" s="5" t="inlineStr">
         <is>
-          <t>17:20-17:30</t>
+          <t>17:30-17:40</t>
         </is>
       </c>
       <c r="B106" s="7" t="n">
@@ -1520,7 +1520,7 @@
     <row r="107" ht="14" customHeight="1">
       <c r="A107" s="5" t="inlineStr">
         <is>
-          <t>17:30-17:40</t>
+          <t>17:40-17:50</t>
         </is>
       </c>
       <c r="B107" s="7" t="n">
@@ -1530,7 +1530,7 @@
     <row r="108" ht="14" customHeight="1">
       <c r="A108" s="5" t="inlineStr">
         <is>
-          <t>17:40-17:50</t>
+          <t>17:50-18:00</t>
         </is>
       </c>
       <c r="B108" s="7" t="n">
@@ -1540,7 +1540,7 @@
     <row r="109" ht="14" customHeight="1">
       <c r="A109" s="5" t="inlineStr">
         <is>
-          <t>17:50-18:00</t>
+          <t>18:00-18:10</t>
         </is>
       </c>
       <c r="B109" s="7" t="n">
@@ -1550,7 +1550,7 @@
     <row r="110" ht="14" customHeight="1">
       <c r="A110" s="5" t="inlineStr">
         <is>
-          <t>18:00-18:10</t>
+          <t>18:10-18:20</t>
         </is>
       </c>
       <c r="B110" s="7" t="n">
@@ -1560,7 +1560,7 @@
     <row r="111" ht="14" customHeight="1">
       <c r="A111" s="5" t="inlineStr">
         <is>
-          <t>18:10-18:20</t>
+          <t>18:20-18:30</t>
         </is>
       </c>
       <c r="B111" s="7" t="n">
@@ -1570,7 +1570,7 @@
     <row r="112" ht="14" customHeight="1">
       <c r="A112" s="5" t="inlineStr">
         <is>
-          <t>18:20-18:30</t>
+          <t>18:30-18:40</t>
         </is>
       </c>
       <c r="B112" s="7" t="n">
@@ -1580,7 +1580,7 @@
     <row r="113" ht="14" customHeight="1">
       <c r="A113" s="5" t="inlineStr">
         <is>
-          <t>18:30-18:40</t>
+          <t>18:40-18:50</t>
         </is>
       </c>
       <c r="B113" s="7" t="n">
@@ -1590,7 +1590,7 @@
     <row r="114" ht="14" customHeight="1">
       <c r="A114" s="5" t="inlineStr">
         <is>
-          <t>18:40-18:50</t>
+          <t>18:50-19:00</t>
         </is>
       </c>
       <c r="B114" s="7" t="n">
@@ -1600,7 +1600,7 @@
     <row r="115" ht="14" customHeight="1">
       <c r="A115" s="5" t="inlineStr">
         <is>
-          <t>18:50-19:00</t>
+          <t>19:00-19:10</t>
         </is>
       </c>
       <c r="B115" s="7" t="n">
@@ -1610,7 +1610,7 @@
     <row r="116" ht="14" customHeight="1">
       <c r="A116" s="5" t="inlineStr">
         <is>
-          <t>19:00-19:10</t>
+          <t>19:10-19:20</t>
         </is>
       </c>
       <c r="B116" s="7" t="n">
@@ -1620,7 +1620,7 @@
     <row r="117" ht="14" customHeight="1">
       <c r="A117" s="5" t="inlineStr">
         <is>
-          <t>19:10-19:20</t>
+          <t>19:20-19:30</t>
         </is>
       </c>
       <c r="B117" s="7" t="n">
@@ -1630,7 +1630,7 @@
     <row r="118" ht="14" customHeight="1">
       <c r="A118" s="5" t="inlineStr">
         <is>
-          <t>19:20-19:30</t>
+          <t>19:30-19:40</t>
         </is>
       </c>
       <c r="B118" s="7" t="n">
@@ -1640,7 +1640,7 @@
     <row r="119" ht="14" customHeight="1">
       <c r="A119" s="5" t="inlineStr">
         <is>
-          <t>19:30-19:40</t>
+          <t>19:40-19:50</t>
         </is>
       </c>
       <c r="B119" s="7" t="n">
@@ -1650,7 +1650,7 @@
     <row r="120" ht="14" customHeight="1">
       <c r="A120" s="5" t="inlineStr">
         <is>
-          <t>19:40-19:50</t>
+          <t>19:50-20:00</t>
         </is>
       </c>
       <c r="B120" s="7" t="n">
@@ -1660,7 +1660,7 @@
     <row r="121" ht="14" customHeight="1">
       <c r="A121" s="5" t="inlineStr">
         <is>
-          <t>19:50-20:00</t>
+          <t>20:00-20:10</t>
         </is>
       </c>
       <c r="B121" s="7" t="n">
@@ -1670,7 +1670,7 @@
     <row r="122" ht="14" customHeight="1">
       <c r="A122" s="5" t="inlineStr">
         <is>
-          <t>20:00-20:10</t>
+          <t>20:10-20:20</t>
         </is>
       </c>
       <c r="B122" s="7" t="n">
@@ -1680,7 +1680,7 @@
     <row r="123" ht="14" customHeight="1">
       <c r="A123" s="5" t="inlineStr">
         <is>
-          <t>20:10-20:20</t>
+          <t>20:20-20:30</t>
         </is>
       </c>
       <c r="B123" s="7" t="n">
@@ -1690,7 +1690,7 @@
     <row r="124" ht="14" customHeight="1">
       <c r="A124" s="5" t="inlineStr">
         <is>
-          <t>20:20-20:30</t>
+          <t>20:30-20:40</t>
         </is>
       </c>
       <c r="B124" s="7" t="n">
@@ -1700,7 +1700,7 @@
     <row r="125" ht="14" customHeight="1">
       <c r="A125" s="5" t="inlineStr">
         <is>
-          <t>20:30-20:40</t>
+          <t>20:40-20:50</t>
         </is>
       </c>
       <c r="B125" s="7" t="n">
@@ -1710,7 +1710,7 @@
     <row r="126" ht="14" customHeight="1">
       <c r="A126" s="5" t="inlineStr">
         <is>
-          <t>20:40-20:50</t>
+          <t>20:50-21:00</t>
         </is>
       </c>
       <c r="B126" s="7" t="n">
@@ -1720,7 +1720,7 @@
     <row r="127" ht="14" customHeight="1">
       <c r="A127" s="5" t="inlineStr">
         <is>
-          <t>20:50-21:00</t>
+          <t>21:00-21:10</t>
         </is>
       </c>
       <c r="B127" s="7" t="n">
@@ -1730,7 +1730,7 @@
     <row r="128" ht="14" customHeight="1">
       <c r="A128" s="5" t="inlineStr">
         <is>
-          <t>21:00-21:10</t>
+          <t>21:10-21:20</t>
         </is>
       </c>
       <c r="B128" s="7" t="n">
@@ -1740,7 +1740,7 @@
     <row r="129" ht="14" customHeight="1">
       <c r="A129" s="5" t="inlineStr">
         <is>
-          <t>21:10-21:20</t>
+          <t>21:20-21:30</t>
         </is>
       </c>
       <c r="B129" s="7" t="n">
@@ -1750,7 +1750,7 @@
     <row r="130" ht="14" customHeight="1">
       <c r="A130" s="5" t="inlineStr">
         <is>
-          <t>21:20-21:30</t>
+          <t>21:30-21:40</t>
         </is>
       </c>
       <c r="B130" s="7" t="n">
@@ -1760,7 +1760,7 @@
     <row r="131" ht="14" customHeight="1">
       <c r="A131" s="5" t="inlineStr">
         <is>
-          <t>21:30-21:40</t>
+          <t>21:40-21:50</t>
         </is>
       </c>
       <c r="B131" s="7" t="n">
@@ -1770,7 +1770,7 @@
     <row r="132" ht="14" customHeight="1">
       <c r="A132" s="5" t="inlineStr">
         <is>
-          <t>21:40-21:50</t>
+          <t>21:50-22:00</t>
         </is>
       </c>
       <c r="B132" s="7" t="n">
@@ -1780,7 +1780,7 @@
     <row r="133" ht="14" customHeight="1">
       <c r="A133" s="5" t="inlineStr">
         <is>
-          <t>21:50-22:00</t>
+          <t>22:00-22:10</t>
         </is>
       </c>
       <c r="B133" s="7" t="n">
@@ -1790,7 +1790,7 @@
     <row r="134" ht="14" customHeight="1">
       <c r="A134" s="5" t="inlineStr">
         <is>
-          <t>22:00-22:10</t>
+          <t>22:10-22:20</t>
         </is>
       </c>
       <c r="B134" s="7" t="n">
@@ -1800,7 +1800,7 @@
     <row r="135" ht="14" customHeight="1">
       <c r="A135" s="5" t="inlineStr">
         <is>
-          <t>22:10-22:20</t>
+          <t>22:20-22:30</t>
         </is>
       </c>
       <c r="B135" s="7" t="n">
@@ -1810,7 +1810,7 @@
     <row r="136" ht="14" customHeight="1">
       <c r="A136" s="5" t="inlineStr">
         <is>
-          <t>22:20-22:30</t>
+          <t>22:30-22:40</t>
         </is>
       </c>
       <c r="B136" s="7" t="n">
@@ -1820,7 +1820,7 @@
     <row r="137" ht="14" customHeight="1">
       <c r="A137" s="5" t="inlineStr">
         <is>
-          <t>22:30-22:40</t>
+          <t>22:40-22:50</t>
         </is>
       </c>
       <c r="B137" s="7" t="n">
@@ -1830,7 +1830,7 @@
     <row r="138" ht="14" customHeight="1">
       <c r="A138" s="5" t="inlineStr">
         <is>
-          <t>22:40-22:50</t>
+          <t>22:50-23:00</t>
         </is>
       </c>
       <c r="B138" s="7" t="n">
@@ -1840,7 +1840,7 @@
     <row r="139" ht="14" customHeight="1">
       <c r="A139" s="5" t="inlineStr">
         <is>
-          <t>22:50-23:00</t>
+          <t>23:00-23:10</t>
         </is>
       </c>
       <c r="B139" s="7" t="n">
@@ -1850,7 +1850,7 @@
     <row r="140" ht="14" customHeight="1">
       <c r="A140" s="5" t="inlineStr">
         <is>
-          <t>23:00-23:10</t>
+          <t>23:10-23:20</t>
         </is>
       </c>
       <c r="B140" s="7" t="n">
@@ -1860,7 +1860,7 @@
     <row r="141" ht="14" customHeight="1">
       <c r="A141" s="5" t="inlineStr">
         <is>
-          <t>23:10-23:20</t>
+          <t>23:20-23:30</t>
         </is>
       </c>
       <c r="B141" s="7" t="n">
@@ -1870,7 +1870,7 @@
     <row r="142" ht="14" customHeight="1">
       <c r="A142" s="5" t="inlineStr">
         <is>
-          <t>23:20-23:30</t>
+          <t>23:30-23:40</t>
         </is>
       </c>
       <c r="B142" s="7" t="n">
@@ -1880,7 +1880,7 @@
     <row r="143" ht="14" customHeight="1">
       <c r="A143" s="5" t="inlineStr">
         <is>
-          <t>23:30-23:40</t>
+          <t>23:40-23:50</t>
         </is>
       </c>
       <c r="B143" s="7" t="n">
@@ -1890,7 +1890,7 @@
     <row r="144" ht="14" customHeight="1">
       <c r="A144" s="5" t="inlineStr">
         <is>
-          <t>23:40-23:50</t>
+          <t>23:50-0:00+1</t>
         </is>
       </c>
       <c r="B144" s="7" t="n">
@@ -1900,11 +1900,11 @@
     <row r="145" ht="14" customHeight="1">
       <c r="A145" s="5" t="inlineStr">
         <is>
-          <t>23:50-24:00</t>
+          <t>0:00+1-0:10+1</t>
         </is>
       </c>
       <c r="B145" s="7" t="n">
-        <v>574.12098</v>
+        <v>907.4543200000001</v>
       </c>
     </row>
   </sheetData>
@@ -1984,7 +1984,7 @@
         <v>750</v>
       </c>
       <c r="C3" t="n">
-        <v>7073.15689</v>
+        <v>6608.24417</v>
       </c>
       <c r="D3" s="6" t="inlineStr">
         <is>
@@ -2002,10 +2002,10 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>4309.167855</v>
+        <v>3559.167855</v>
       </c>
       <c r="C4" t="n">
-        <v>1892.218881</v>
+        <v>2357.131601</v>
       </c>
     </row>
     <row r="5" ht="14" customFormat="1" customHeight="1" s="5">
@@ -2015,7 +2015,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>4757.431665</v>
+        <v>5507.431665</v>
       </c>
       <c r="C5" t="n">
         <v>101.22376</v>
@@ -2031,7 +2031,7 @@
         <v>0</v>
       </c>
       <c r="C6" t="n">
-        <v>6422.36876</v>
+        <v>5631.87428</v>
       </c>
     </row>
     <row r="7" ht="14" customFormat="1" customHeight="1" s="5">
@@ -2044,7 +2044,7 @@
         <v>4800</v>
       </c>
       <c r="C7" t="n">
-        <v>3177.63125</v>
+        <v>3968.12573</v>
       </c>
     </row>
   </sheetData>

</xml_diff>